<commit_message>
Enforce English prompt excerpts and regenerate qualitative gate artifacts
</commit_message>
<xml_diff>
--- a/RQ2_Prompt_Effectiveness_Modeling/results/qualitative/gate0/gate0_qualitative_patterns.xlsx
+++ b/RQ2_Prompt_Effectiveness_Modeling/results/qualitative/gate0/gate0_qualitative_patterns.xlsx
@@ -570,7 +570,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Kotlin の sksamuel/scrimage ライブラリで、画像上に文字列を描画し、文字列の縁取りをするコードを生成してください。文字の色は白、縁は黒で描画します。</t>
+          <t>Using Kotlin with the sksamuel/scrimage library, generate code to draw text on an image with an outline. Render white text with a black border.</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>git diff は違いがあった場合のステータスコードは何でしょうか。ありがとうございます。diffはどうでしょうか。</t>
+          <t>What is the exit status code for git diff when differences are found? Thank you. Also, what about diff?</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>こちらの変更に対して、『VVMファイルからVoiceModelをコンストラクトする。』という表現について、生成・解放などの用語選択に関する意見が交わされました。</t>
+          <t>For this change, there was discussion about the wording 'construct VoiceModel from a VVM file', including terminology choices such as construct versus allocate/free.</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">

</xml_diff>